<commit_message>
Settle rundatetime and workrel in the mapping
rundatetime fills SM36's NOTBEFORE — an earliest-start floor — and
workrel alone decides month-start vs month-end counting. That resolves
the overlap the previous version flagged, and turns up a new gap: APJ has
no NOTBEFORE equivalent, so it gets its own row as 불가 pending whether
the first start timestamp can absorb it.

It also leaves StartRestriction without an AS-IS source. Our API exposes
the holiday-avoidance code but no create parameter maps to it unless
workrel's value doubles as EXECUTE_BEFORE, which its name suggests but
nothing confirms. Noted on the mapping sheet and in the checks.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rKnPQ2EVBywDqfgn5AEBx
</commit_message>
<xml_diff>
--- a/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
+++ b/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="377">
   <si>
     <r>
       <rPr>
@@ -3024,7 +3024,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">값 도메인 확인됨</t>
+      <t xml:space="preserve">값 도메인은 확인됨</t>
     </r>
     <r>
       <rPr>
@@ -3058,24 +3058,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">의 어느 필드가 이 자리인지는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">workrel / rundatetime </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">중 확인이 필요하다</t>
+      <t xml:space="preserve">파라미터 중 이 자리에 오는 것이 없다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">workrel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EXECUTE_BEFORE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 함께 가는지 확인 필요</t>
     </r>
   </si>
   <si>
@@ -3182,6 +3199,40 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">workrel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값 유무가 이 판정이다 — 확인됨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다만 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">APJ </t>
     </r>
     <r>
@@ -3207,7 +3258,79 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">는 추측이다</t>
+      <t xml:space="preserve">는 추측이라 첫 테스트의 실행 예정일로 확정해야 한다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지정 시각 전에는 실행 금지 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(rundatetime)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NOTBEFORE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자리다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 대응 필드가 없다</t>
     </r>
     <r>
       <rPr>
@@ -3224,7 +3347,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">첫 테스트의 실행 예정일로 판정해야 한다</t>
+      <t xml:space="preserve">첫 시작 시각이 그 하한을 겸할 수 있는지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회차마다 걸리는 값인지 확인이 필요하다</t>
     </r>
   </si>
   <si>
@@ -5840,37 +5980,379 @@
     <t xml:space="preserve">실행관련시간</t>
   </si>
   <si>
-    <t xml:space="preserve">?</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월초 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">말일 판정에 쓰인다고 봤는데 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
+    <t xml:space="preserve">대응 없음</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NOTBEFORE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 들어간다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 시각 전에는 돌리지 마라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 하한이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 같은 필드가 없다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">첫 시작 시각</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(START_INFO-timestamp)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 그 역할을 겸하는지 확인 필요</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">workrel</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">excutbefor </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타입</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTH_INFO-shift_direction</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값이 있으면 월초부터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">없으면 말일부터 센다 — 확인됨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값 자체가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EXECUTE_BEFORE(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">휴일 회피</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로도 가는지는 확인 필요</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 표시 두 곳이 새로 확인된 것이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. jobuser </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 되는 것으로 판정이 바뀌었고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, repcycle </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 우리 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">API </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">형태를 바꿔야 한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">우리 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">API </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">StartRestriction </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 대응 필드가 없다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -5879,254 +6361,12 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">과 역할이 겹친다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">둘 중 무엇이 무엇을 채우는지 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AS-IS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">코드로 확정해야 한다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">workrel</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">excutbefor </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">타입</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">StartRestriction / CountFromEnd</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">EXCEPTION-start_restriction_code
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">또는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MONTH_INFO-shift_direction</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AS-IS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로직상 이 값 유무로 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">BOFMONTH / EOFMONTH </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가 갈린다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">세는 방향</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">). EXECUTE_BEFORE(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">휴일 회피</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로도 쓰이는지 확인 필요</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">★ 표시 두 곳이 이번에 새로 확인된 것이다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. jobuser </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 되는 것으로 판정이 바뀌었고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, repcycle </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 우리 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">API </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">형태를 바꿔야 한다</t>
+      <t xml:space="preserve">값이 그 자리인지 확인이 필요하다</t>
     </r>
     <r>
       <rPr>
@@ -7827,42 +8067,25 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">rundatetime / workrel </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">중 어느 쪽이 월초</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">말일을 가르나</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">둘이 역할이 겹쳐 보인다</t>
+      <t xml:space="preserve">NOTBEFORE(rundatetime) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 첫 회만 걸리나 회차마다 걸리나</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">첫 회뿐이면 시작 시각으로 흡수된다</t>
     </r>
     <r>
       <rPr>
@@ -7879,8 +8102,125 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">잘못 매핑하면 실행일이 통째로 어긋난다</t>
-    </r>
+      <t xml:space="preserve">회차마다면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 표현할 방법이 없다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">workrel </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">EXECUTE_BEFORE(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">휴일 회피</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로도 들어가나</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아니면 우리 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">StartRestriction </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 넣을 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값이 없다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">중간</t>
   </si>
   <si>
     <r>
@@ -7961,9 +8301,6 @@
       </rPr>
       <t xml:space="preserve">필요하면 파라미터를 추가해야 한다</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">중간</t>
   </si>
   <si>
     <t xml:space="preserve">운영 데이터</t>
@@ -9711,7 +10048,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="n">
-        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$33,$A12)</f>
+        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$34,$A12)</f>
         <v>15</v>
       </c>
       <c r="E12" s="8" t="s">
@@ -9723,7 +10060,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="7" t="n">
-        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$33,$A13)</f>
+        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$34,$A13)</f>
         <v>6</v>
       </c>
       <c r="E13" s="8" t="s">
@@ -9735,8 +10072,8 @@
         <v>15</v>
       </c>
       <c r="B14" s="7" t="n">
-        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$33,$A14)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('2.기능판정'!$C$4:$C$34,$A14)</f>
+        <v>10</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>16</v>
@@ -9748,7 +10085,7 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">SUM(B12:B14)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>18</v>
@@ -10132,7 +10469,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -10305,7 +10642,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
         <v>116</v>
       </c>
@@ -10322,9 +10659,9 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>129</v>
@@ -10341,33 +10678,33 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>132</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="B15" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="23" t="s">
         <v>135</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="22" t="s">
-        <v>114</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>136</v>
@@ -10375,109 +10712,109 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="C16" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16" s="11" t="s">
         <v>138</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E17" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="E17" s="22" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>145</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="B19" s="22" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="B19" s="22" t="s">
+      <c r="C19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="22" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="11" t="s">
+      <c r="C20" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="11" t="s">
         <v>151</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="E21" s="22" t="s">
         <v>154</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>156</v>
@@ -10485,8 +10822,8 @@
       <c r="C22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>114</v>
+      <c r="D22" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>157</v>
@@ -10494,7 +10831,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B23" s="22" t="s">
         <v>158</v>
@@ -10503,32 +10840,32 @@
         <v>15</v>
       </c>
       <c r="D23" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="22" t="s">
         <v>159</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="E24" s="11" t="s">
         <v>162</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B25" s="22" t="s">
         <v>164</v>
@@ -10543,9 +10880,9 @@
         <v>165</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>166</v>
@@ -10553,93 +10890,93 @@
       <c r="C26" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E26" s="11" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B27" s="22" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
+      <c r="C27" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="E27" s="23" t="s">
         <v>170</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="B29" s="22" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="B29" s="22" t="s">
+      <c r="C29" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="E29" s="23" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="E29" s="23" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B30" s="8" t="s">
+      <c r="D30" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="E30" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
-        <v>172</v>
-      </c>
-      <c r="B31" s="22" t="s">
+      <c r="D31" s="23" t="s">
         <v>182</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>114</v>
       </c>
       <c r="E31" s="23" t="s">
         <v>183</v>
@@ -10647,36 +10984,53 @@
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
+      <c r="D33" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="E33" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="C33" s="9" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D33" s="22" t="s">
-        <v>189</v>
-      </c>
-      <c r="E33" s="22" t="s">
-        <v>190</v>
+      <c r="D34" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -10708,226 +11062,226 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>11</v>
@@ -10936,56 +11290,56 @@
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B15" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>248</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>243</v>
-      </c>
       <c r="F15" s="23" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>118</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>11</v>
@@ -10994,87 +11348,87 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>201</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="F19" s="22" t="s">
-        <v>264</v>
+        <v>203</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>267</v>
+        <v>127</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="F20" s="11" t="s">
         <v>269</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
@@ -11113,25 +11467,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C5" s="18"/>
       <c r="D5" s="18"/>
@@ -11139,10 +11493,10 @@
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -11150,10 +11504,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C7" s="18"/>
       <c r="D7" s="18"/>
@@ -11161,167 +11515,167 @@
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="29" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="8" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
       <c r="E20" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="29" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
       <c r="E21" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -11330,7 +11684,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B24" s="31"/>
       <c r="C24" s="31"/>
@@ -11339,7 +11693,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -11374,7 +11728,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -11385,12 +11739,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11398,130 +11752,130 @@
         <v>38</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B5" s="23" t="s">
+        <v>332</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>333</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>331</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>332</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
+        <v>328</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>337</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>338</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>337</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>338</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="B8" s="11" t="s">
         <v>339</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="B8" s="8" t="s">
         <v>340</v>
       </c>
+      <c r="C8" s="11" t="s">
+        <v>341</v>
+      </c>
       <c r="D8" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>342</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>335</v>
+        <v>343</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>343</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>344</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
+        <v>339</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>346</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>347</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>345</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>346</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>348</v>
@@ -11529,8 +11883,8 @@
       <c r="C12" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>330</v>
+      <c r="D12" s="9" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11540,151 +11894,165 @@
       <c r="B13" s="22" t="s">
         <v>351</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>352</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>335</v>
+      <c r="D13" s="10" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>355</v>
-      </c>
-      <c r="C15" s="22" t="s">
         <v>356</v>
       </c>
+      <c r="C15" s="23" t="s">
+        <v>357</v>
+      </c>
       <c r="D15" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>357</v>
-      </c>
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>358</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="8" t="s">
         <v>359</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D16" s="9" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B17" s="23" t="s">
+        <v>361</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>362</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="C17" s="22" t="s">
-        <v>361</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>357</v>
-      </c>
       <c r="B18" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>357</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>364</v>
+        <v>360</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>365</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>365</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>366</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>357</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>366</v>
+        <v>360</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>367</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a sheet comparing the AS-IS RFCs with the APJ API calls
Two tables: each AS-IS function mapped to the APJ call that replaces it,
and the APJ method list split by whether we call it.

The mapping is not one-to-one in two places. CHANGE needs two calls
because no modify method was found, which is why jobname changes; and
STATUS has a different shape entirely — the AS-IS RFC selects TBTCO by
job name and status with a date range, while GET_JOB_STATUS reads exactly
one job by name and count.

GET_JOB_DETAIL is listed as available but unused: it returns the job's
definition, not just its status, which is what a change screen would need
to prefill. Job modify, job list and job log methods are listed as
unconfirmed rather than absent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rKnPQ2EVBywDqfgn5AEBx
</commit_message>
<xml_diff>
--- a/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
+++ b/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
@@ -11,6 +11,7 @@
     <sheet name="1.개념비교" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="2.SM36파라미터" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="3.APJ파라미터" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="4.API비교" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="307">
   <si>
     <t xml:space="preserve">SM36 / SM37  vs  Application Job</t>
   </si>
@@ -4078,6 +4079,1601 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">를 한 번 훑어보는 것이 좋다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS RFC </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기능  ↔  </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Application Job API</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배치 인터페이스 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개가 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 어느 호출로 바뀌는지</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그리고 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ API </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전체 목록</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">① AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기능 → </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호출</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">AS-IS RFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기능</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">호출</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">호출 수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">차이점</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZBC_BATCH_JOB_CREATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 생성</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">화면을 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BDC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JOB_OPEN → JOB_SUBMIT → JOB_CLOSE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">까지 돌린다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 시작조건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반복조건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파라미터를 한 번에 넘기고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname / jobcount </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 받는다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ZBC_BATCH_JOB_CHANGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 변경</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANCEL_JOB + SCHEDULE_JOB</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">★ APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 수정 메서드를 못 찾아 취소하고 다시 건다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그래서 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname / jobcount </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 바뀐다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수정 메서드가 있으면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회로 줄고 식별자도 유지된다 — 확인 필요</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ZBC_BATCH_JOB_DELETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 삭제</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANCEL_JOB</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">삭제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">", APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">취소</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">취소된 잡은 사라지지 않고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Cancelled </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">상태로 남는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이력을 지우고 싶으면 별도 처리가 필요하다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ZBC_BATCH_JOB_STATUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상태 조회</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET_JOB_STATUS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 모양이 다르다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TBTCO </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">상태</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(P </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예정 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">릴리스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SELECT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해서 여러 건을 잡고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실제로는 첫 건만 반환</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기간 조건도 받는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname + jobcount </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 정확히 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건을 읽는다 — 기간 검색이 안 된다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">② APJ API </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메서드</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메서드</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">무엇을 하나</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대응</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">쓰고 있는 것</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡을 새로 건다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREATE</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시작조건 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반복조건 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파라미터를 한 번에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. jobname / jobcount </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 돌려준다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡을 끊는다 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이후 회차 포함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">DELETE</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 내부에서 커밋한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. RAP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">트랜잭션 안에서 부르면 덤프가 나므로 별도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">LUW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 불러야 한다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건의 현재 상태</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">STATUS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname + jobcount </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">상태값 도메인은 아직 미검증</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">있는데 안 쓰는 것</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET_JOB_DETAIL</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">건의 정의까지 읽는다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 상태뿐 아니라 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무슨 조건으로 걸렸는지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파라미터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스케줄 조건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 읽을 수 있다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">변경 화면에서 기존 값을 채워 보여줄 때 쓸 만하다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">있는지 확인이 필요한 것</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 수정 메서드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">건 잡의 조건을 바꾼다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHANGE</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있으면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">changeJob </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회 호출로 줄고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">jobname </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 안 바뀐다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">연동 영향이 가장 큰 항목</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 목록 조회 메서드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">조건으로 여러 건을 찾는다</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">STATUS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 기간 검색</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있으면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AS-IS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 기간 검색을 그대로 살릴 수 있다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">잡 로그 조회 메서드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실행 로그를 읽는다</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 로그는 앱에서는 보이는데 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">API </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 읽는 방법이 있는지 확인이 필요하다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메서드 목록은 확인된 것만 적었다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. CL_APJ_RT_API </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ADT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에서 열어 나머지를 채우는 것이 좋다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">iv_username </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">it_job_parameter_value_simple </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 그랬듯 뒤늦게 나오는 것이 있다</t>
     </r>
     <r>
       <rPr>
@@ -4099,7 +5695,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4210,6 +5806,19 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -4304,7 +5913,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4378,6 +5987,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6022,4 +7635,298 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="54"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15"/>
+      <c r="B14" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15"/>
+      <c r="B15" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15"/>
+      <c r="B16" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15"/>
+      <c r="B18" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15"/>
+      <c r="B20" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15"/>
+      <c r="B21" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15"/>
+      <c r="B22" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A24:E24"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correct what the simple parameter table actually is
I had described it_job_parameter_value_simple as a name/value pair list.
It is step_nr + name + t_value, so it still carries a value table and
ranges are expressible. "Simple" means it omits the parameter metadata,
not that the values are scalars.

That matters because the JSON shape our adapter already documents —
name plus t_value — is the simple structure, while the code declares the
non-simple type. Softened the non-simple row to say its layout is
unconfirmed rather than asserting a field list I had inferred.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rKnPQ2EVBywDqfgn5AEBx
</commit_message>
<xml_diff>
--- a/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
+++ b/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
@@ -3014,123 +3014,160 @@
     <t xml:space="preserve">it_job_parameter_value</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프로그램에 넘길 값 — </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SAP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">레인지 형식</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">selname / kind / sign / option / low / high </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로 넣는다</t>
+    <t xml:space="preserve">프로그램에 넘길 값</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">행 구조 미확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. _simple </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보다 파라미터 종류</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타입 같은 메타 정보를 더 요구하는 것으로 보인다</t>
     </r>
   </si>
   <si>
     <t xml:space="preserve">it_job_parameter_value_simple</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프로그램에 넘길 값 — 이름 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">값</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">★ 외부에서 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">JSON </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">으로 받을 때 이쪽이 훨씬 단순하다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">레인지가 필요 없으면 이걸 쓴다</t>
+    <t xml:space="preserve">프로그램에 넘길 값 — 메타 정보 없이</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">★ step_nr + name + t_value </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세 필드뿐이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. t_value </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 그대로 들고 있어 레인지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(BT, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다중 선택</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 표현된다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 값이 단순하다는 뜻이 아니라 파라미터 정의를 잡 카탈로그에서 가져다 쓴다는 뜻이다</t>
     </r>
   </si>
   <si>
@@ -6211,7 +6248,7 @@
       <c r="E41" s="15"/>
       <c r="F41" s="15"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="5" t="s">
         <v>162</v>
@@ -6225,14 +6262,14 @@
       <c r="E42" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="F42" s="5" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
-      <c r="B43" s="17" t="s">
-        <v>69</v>
+      <c r="B43" s="5" t="s">
+        <v>162</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>166</v>
@@ -6243,7 +6280,7 @@
       <c r="E43" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" s="6" t="s">
         <v>168</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Close the multi-step question
A job catalog entry holds exactly one execution class, a template points
at one entry, and SCHEDULE_JOB takes one template name — so nothing in
the call could say what a second step would run. step_nr existing does
not reopen it; the field is there because the same structure reads
classic jobs, which do have several steps.

Recorded the chain on the multi-step row instead of the "confirm whether
a template can define steps" note, and said plainly what sequencing
inside one class costs: no per-step status, log, or restart. The step_nr
row now states it is always 1 when scheduling.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rKnPQ2EVBywDqfgn5AEBx
</commit_message>
<xml_diff>
--- a/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
+++ b/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="234">
   <si>
     <t xml:space="preserve">SM36 / SM37  vs  Application Job</t>
   </si>
@@ -1355,6 +1355,749 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 하나에 프로그램 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개를 순서대로</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 카탈로그 엔트리가 실행 클래스를 하나만 갖는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿도 엔트리 하나</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, SCHEDULE_JOB </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 템플릿명 하나라 스텝 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 실행 대상을 정의할 자리가 없다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실행 클래스 안에서 순서대로 부르면 결과는 같지만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스텝별 상태</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로그</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재시작은 못 한다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프로그램 타입 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(ABAP / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">외부 명령 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">외부 프로그램</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">실행 클래스만</t>
+  </si>
+  <si>
+    <t xml:space="preserve">무엇을 실행할지</t>
+  </si>
+  <si>
+    <t xml:space="preserve">외부 명령과 외부 프로그램은 아예 없다</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ABAP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프로그램명</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">iv_job_template_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실행 대상 지정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿 → 잡 카탈로그 엔트리 → 실행 클래스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">런타임에 이름을 넘기지 않고 미리 등록한다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">배리언트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">선택 화면 값 묶음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">템플릿이 배리언트 자리다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배리언트 언어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">텍스트 언어</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스텝 사용자 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Step user)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">iv_username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어떤 권한으로 돌릴지</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 테스트 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. TBTCO-AUTHCKNAM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 들어간다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. RELUNAME </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에 호출 계정이 남는 건 정상</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">인쇄 파라미터 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아카이빙</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">출력 장치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보관</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">스풀이 없어 해당 없음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">시작 조건</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">즉시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Immediate)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">START_INFO-start_immediately</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바로 실행</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">날짜 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시간</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">START_INFO-timestamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">예약 실행</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">UTC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타임스탬프다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 보내면 오류라 즉시 실행이어도 현재 시각을 채운다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">최종 시작 시각 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(No start after)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">END_INFO type = BY + timestamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이 시각 넘으면 시작 안 함</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">돌고 있는 잡은 안 끊는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. type </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BY </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 아직 미검증</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선행 잡 종료 후 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(After job)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">다른 잡이 끝나면 기동</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡 체이닝이 없다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">한 클래스로 묶거나 별도 설계가 필요하다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이벤트 발생 시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(After event)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이벤트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ID + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파라미터로 기동</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">이벤트로 도는 배치가 있으면 설계를 바꿔야 한다</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오퍼레이션 모드 전환 시</t>
+  </si>
+  <si>
+    <t xml:space="preserve">모드가 바뀌면 기동</t>
+  </si>
+  <si>
+    <t xml:space="preserve">반복 주기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주기 단위 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -1367,70 +2110,252 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">파라미터 구조의 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">step_nr)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">잡 하나에 프로그램 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개를 순서대로</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">★ 파라미터 값 테이블이 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">step_nr </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">을 나른다 — 스텝 개념 자체는 살아 있다</t>
+      <t xml:space="preserve">분 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">주 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHEDULING_INFO-periodic_granularity + periodic_value</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">몇 분</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일마다 돌지</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단위 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">값 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">라 모양이 같다</t>
     </r>
     <r>
       <rPr>
@@ -1447,7 +2372,256 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">잡 템플릿이 스텝을 여럿 정의할 수 있는지 확인 필요</t>
+      <t xml:space="preserve">단위 값 도메인은 미검증</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여러 단위 합산 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개월 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ 15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= 45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">합산 주기</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PRD* </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필드를 더한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 단위를 하나만 고를 수 있다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHEDULING_INFO-timezone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">반복 계산의 기준 타임존</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 시스템 시간 고정이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. APJ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 나은 점</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">END_INFO type = AFTER + max_iterations</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">N </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회 실행 후 종료</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHEDULING_INFO-weekday_info</t>
+  </si>
+  <si>
+    <t xml:space="preserve">요일 지정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매주 화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">처럼 한 잡에 요일을 여럿</t>
     </r>
     <r>
       <rPr>
@@ -1464,34 +2638,164 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">안 되면 실행 클래스 안에서 순차 호출</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프로그램 타입 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(ABAP / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">외부 명령 </t>
+      <t xml:space="preserve">구조는 미확인</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTH_INFO-week_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">몇 번째 주</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">weekday_info </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와 묶으면 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매월 둘째 주 화요일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">제한 조건</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공장달력 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ID</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">EXCEPTION-calendar_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작업일 판단의 기준 달력</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작업일 번호 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Workday no.)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTH_INFO-day + use_working_days_ind</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그 달의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">n </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">번째 작업일</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM36 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 공장달력이 있으면 항상 작업일 기준이라 별도 플래그가 없다</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월초부터 </t>
     </r>
     <r>
       <rPr>
@@ -1508,7 +2812,351 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">외부 프로그램</t>
+      <t xml:space="preserve">말일부터 세기</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MONTH_INFO-shift_direction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작업일을 어느 쪽에서 셀지</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NUMC(2) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">인데 도메인 고정값이 없다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 01 / 02 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 추측이라 첫 테스트로 확정해야 한다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">비근무일 처리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXCEPTION-start_restriction_code</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">휴일이면 앞당김 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미룸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미실행 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그대로</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">D </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미실행 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ B </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">앞당김 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ A </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미룸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ N </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그대로</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Not before</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이 시각 전에는 실행 금지</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">★ 대응이 없다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">첫 시작 시각이 하한을 겸할 수 있는지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회차마다 걸리는 값인지 확인 필요</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">파라미터 전달</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배리언트 값</t>
+  </si>
+  <si>
+    <t xml:space="preserve">it_job_parameter_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프로그램에 넘길 값</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">행 구조 미확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. _simple </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보다 파라미터 종류</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타입 같은 메타 정보를 더 요구하는 것으로 보인다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">it_job_parameter_value_simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프로그램에 넘길 값 — 메타 정보 없이</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">★ step_nr + name + t_value </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세 필드뿐이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. t_value </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 그대로 들고 있어 레인지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(BT, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">다중 선택</t>
     </r>
     <r>
       <rPr>
@@ -1519,49 +3167,83 @@
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">실행 클래스만</t>
-  </si>
-  <si>
-    <t xml:space="preserve">무엇을 실행할지</t>
-  </si>
-  <si>
-    <t xml:space="preserve">외부 명령과 외부 프로그램은 아예 없다</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ABAP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프로그램명</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">iv_job_template_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실행 대상 지정</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">템플릿 → 잡 카탈로그 엔트리 → 실행 클래스</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도 표현된다 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단순</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 값이 단순하다는 뜻이 아니라 파라미터 정의를 잡 카탈로그에서 가져다 쓴다는 뜻이다</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">스텝별 배리언트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">step_nr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이 값이 붙을 스텝 번호</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">잡을 걸 때는 항상 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이다 — 스텝이 하나뿐이라 다른 값이 나올 수 없다</t>
     </r>
     <r>
       <rPr>
@@ -1578,229 +3260,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">런타임에 이름을 넘기지 않고 미리 등록한다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">배리언트</t>
-  </si>
-  <si>
-    <t xml:space="preserve">선택 화면 값 묶음</t>
-  </si>
-  <si>
-    <t xml:space="preserve">템플릿이 배리언트 자리다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">배리언트 언어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">텍스트 언어</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">스텝 사용자 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Step user)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">iv_username</t>
-  </si>
-  <si>
-    <t xml:space="preserve">어떤 권한으로 돌릴지</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">★ 테스트 확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. TBTCO-AUTHCKNAM </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">에 들어간다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. RELUNAME </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">에 호출 계정이 남는 건 정상</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">인쇄 파라미터 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">아카이빙</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">출력 장치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">매수</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보관</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">스풀이 없어 해당 없음</t>
-  </si>
-  <si>
-    <t xml:space="preserve">시작 조건</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">즉시 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Immediate)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">START_INFO-start_immediately</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바로 실행</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">날짜 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시간</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">START_INFO-timestamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">예약 실행</t>
-  </si>
-  <si>
+      <t xml:space="preserve">필드가 있는 것은 </t>
+    </r>
     <r>
       <rPr>
         <sz val="10"/>
@@ -1816,244 +3277,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">UTC </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">타임스탬프다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. 0 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">을 보내면 오류라 즉시 실행이어도 현재 시각을 채운다</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">최종 시작 시각 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(No start after)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">END_INFO type = BY + timestamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이 시각 넘으면 시작 안 함</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">돌고 있는 잡은 안 끊는다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. type </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">값 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">BY </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 아직 미검증</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">선행 잡 종료 후 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(After job)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">다른 잡이 끝나면 기동</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">잡 체이닝이 없다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">한 클래스로 묶거나 별도 설계가 필요하다</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이벤트 발생 시 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(After event)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이벤트 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ID + </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">파라미터로 기동</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">이벤트로 도는 배치가 있으면 설계를 바꿔야 한다</t>
-  </si>
-  <si>
-    <t xml:space="preserve">오퍼레이션 모드 전환 시</t>
-  </si>
-  <si>
-    <t xml:space="preserve">모드가 바뀌면 기동</t>
-  </si>
-  <si>
-    <t xml:space="preserve">반복 주기</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주기 단위 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">값 </t>
+      <t xml:space="preserve">밖에서 만든 클래식 잡</t>
     </r>
     <r>
       <rPr>
@@ -2070,75 +3294,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">분 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월</t>
+      <t xml:space="preserve">스텝 여럿</t>
     </r>
     <r>
       <rPr>
@@ -2149,1061 +3305,13 @@
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">SCHEDULING_INFO-periodic_granularity + periodic_value</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">몇 분</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일마다 돌지</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SM36 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">APJ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단위 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">값 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">" </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">라 모양이 같다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단위 값 도메인은 미검증</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">여러 단위 합산 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개월 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ 15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= 45</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">합산 주기</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SM36 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PRD* </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">필드를 더한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. APJ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 단위를 하나만 고를 수 있다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">SCHEDULING_INFO-timezone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">반복 계산의 기준 타임존</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SM36 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 시스템 시간 고정이다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. APJ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가 나은 점</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">END_INFO type = AFTER + max_iterations</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">N </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">회 실행 후 종료</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">SCHEDULING_INFO-weekday_info</t>
-  </si>
-  <si>
-    <t xml:space="preserve">요일 지정</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">매주 화</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">목</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">" </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">처럼 한 잡에 요일을 여럿</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">구조는 미확인</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">MONTH_INFO-week_number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">몇 번째 주</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">weekday_info </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">와 묶으면 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">매월 둘째 주 화요일</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">제한 조건</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공장달력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ID</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">EXCEPTION-calendar_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">작업일 판단의 기준 달력</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">작업일 번호 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Workday no.)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">MONTH_INFO-day + use_working_days_ind</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그 달의 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">n </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">번째 작업일</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SM36 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 공장달력이 있으면 항상 작업일 기준이라 별도 플래그가 없다</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월초부터 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">말일부터 세기</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">MONTH_INFO-shift_direction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">작업일을 어느 쪽에서 셀지</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NUMC(2) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">인데 도메인 고정값이 없다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. 01 / 02 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 추측이라 첫 테스트로 확정해야 한다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">비근무일 처리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXCEPTION-start_restriction_code</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">휴일이면 앞당김 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미룸 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미실행 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그대로</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">D </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미실행 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ B </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">앞당김 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ A </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">미룸 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ N </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그대로</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Not before</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이 시각 전에는 실행 금지</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">★ 대응이 없다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">첫 시작 시각이 하한을 겸할 수 있는지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">회차마다 걸리는 값인지 확인 필요</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">파라미터 전달</t>
-  </si>
-  <si>
-    <t xml:space="preserve">배리언트 값</t>
-  </si>
-  <si>
-    <t xml:space="preserve">it_job_parameter_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">프로그램에 넘길 값</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">행 구조 미확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. _simple </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보다 파라미터 종류</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">타입 같은 메타 정보를 더 요구하는 것으로 보인다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">it_job_parameter_value_simple</t>
-  </si>
-  <si>
-    <t xml:space="preserve">프로그램에 넘길 값 — 메타 정보 없이</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">★ step_nr + name + t_value </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">세 필드뿐이다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. t_value </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">를 그대로 들고 있어 레인지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(BT, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">다중 선택</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도 표현된다 — </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단순</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">" </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 값이 단순하다는 뜻이 아니라 파라미터 정의를 잡 카탈로그에서 가져다 쓴다는 뜻이다</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">스텝별 배리언트</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step_nr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이 값이 붙을 스텝 번호</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">스텝이 하나면 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이다</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 읽을 때 같은 구조를 쓰기 때문으로 보인다</t>
     </r>
     <r>
       <rPr>
@@ -5786,88 +5894,88 @@
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
     </row>
-    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>81</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>54</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>89</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16"/>
       <c r="B17" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>55</v>
@@ -5877,42 +5985,42 @@
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16"/>
       <c r="B19" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E20" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -5923,13 +6031,13 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>53</v>
@@ -5939,85 +6047,85 @@
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16"/>
       <c r="B24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E26" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16"/>
       <c r="B27" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C27" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>55</v>
@@ -6026,7 +6134,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -6037,37 +6145,37 @@
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>126</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C30" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E30" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6076,16 +6184,16 @@
         <v>69</v>
       </c>
       <c r="C31" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="E31" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6094,10 +6202,10 @@
         <v>69</v>
       </c>
       <c r="C32" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="E32" s="13" t="s">
         <v>56</v>
@@ -6110,16 +6218,16 @@
         <v>69</v>
       </c>
       <c r="C33" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>137</v>
       </c>
       <c r="E33" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6128,21 +6236,21 @@
         <v>69</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="E34" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -6153,13 +6261,13 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="D36" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>53</v>
@@ -6169,78 +6277,78 @@
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="D37" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16"/>
       <c r="B38" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="D38" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="E38" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16"/>
       <c r="B39" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="D39" s="5" t="s">
         <v>155</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C40" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E40" s="12" t="s">
         <v>55</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -6251,60 +6359,60 @@
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="D42" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="E42" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D43" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="E43" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="D44" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>171</v>
       </c>
       <c r="E44" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -6318,16 +6426,16 @@
         <v>69</v>
       </c>
       <c r="C46" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D46" s="5" t="s">
         <v>174</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>175</v>
       </c>
       <c r="E46" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -6366,107 +6474,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="6" t="s">
         <v>188</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="E7" s="6" t="s">
         <v>193</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>197</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6474,13 +6582,13 @@
         <v>2</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>205</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>206</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>62</v>
@@ -6488,7 +6596,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
@@ -6498,51 +6606,51 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>212</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>215</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -6552,21 +6660,21 @@
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -6576,51 +6684,51 @@
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="5" t="s">
         <v>225</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>

</xml_diff>

<commit_message>
Reopen the multi-step verdict
The ADT documentation for it_job_parameter_value_simple says it is for
scheduling a job made of several steps, with step_nr as the step number.
That outweighs the chain I closed the question with, which had a gap: a
catalog entry holding one class is confirmed, but a template holding one
entry was my inference, not a finding. If a template can bundle several
entries, the documentation and the structure agree and multi-step
carries over.

Added a 확인중 verdict rather than flipping the row to 가능 — that would
repeat the same mistake in the other direction. The row now names the one
check that settles it: try adding a second step in job template
maintenance.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rKnPQ2EVBywDqfgn5AEBx
</commit_message>
<xml_diff>
--- a/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
+++ b/abap/zbc_job/SM36_vs_ApplicationJob.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="271">
   <si>
     <t xml:space="preserve">한 장 총정리 — 제일 큰 차이</t>
   </si>
@@ -210,66 +210,59 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">잡 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">실행 클래스 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">클래스 안에서 순서대로 부르면 결과는 같다</t>
+    <t xml:space="preserve">확인 중 — 템플릿이 스텝을 여럿 가질 수 있나</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SAP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">문서가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여러 단계로 이루어진 작업</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">을 명시한다</t>
     </r>
     <r>
       <rPr>
@@ -286,7 +279,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">대신 스텝별 상태</t>
+      <t xml:space="preserve">되면 그대로 넘어가고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안 되면 클래스 안에서 순차 호출 — 그 경우 스텝별 상태</t>
     </r>
     <r>
       <rPr>
@@ -1757,7 +1767,76 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">스텝은 클래스 안에서 순서대로 부르는 것으로 바꾼다</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인 중 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">템플릿이 스텝을 여럿 갖는지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SAP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">문서가 다단계 작업을 언급한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안 되면 클래스 안에서 순차 호출로 바꾼다</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">잡 식별</t>
@@ -2150,6 +2229,9 @@
     <t xml:space="preserve">추가</t>
   </si>
   <si>
+    <t xml:space="preserve">확인중</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="9"/>
@@ -2309,7 +2391,45 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">에만 있다</t>
+      <t xml:space="preserve">에만 있다  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인중 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아직 판정 못 함</t>
     </r>
   </si>
   <si>
@@ -2555,6 +2675,42 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">잡 템플릿 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인 중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">잡 하나에 프로그램 </t>
     </r>
     <r>
@@ -2579,10 +2735,70 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">잡 카탈로그 엔트리가 실행 클래스를 하나만 갖는다</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">★ it_job_parameter_value_simple </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ADT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설명이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">여러 단계로 이루어진 작업을 예약할 때</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">라고 명시한다</t>
     </r>
     <r>
       <rPr>
@@ -2599,24 +2815,75 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">템플릿도 엔트리 하나</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, SCHEDULE_JOB </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도 템플릿명 하나라 스텝 </t>
+      <t xml:space="preserve">확인된 것은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">카탈로그 엔트리 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">클래스 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">까지이고 템플릿이 엔트리를 여럿 묶을 수 있는지는 미확인 — 잡 템플릿 생성 화면에서 스텝을 </t>
     </r>
     <r>
       <rPr>
@@ -2633,7 +2900,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">의 실행 대상을 정의할 자리가 없다</t>
+      <t xml:space="preserve">개 넣어보면 판정된다</t>
     </r>
     <r>
       <rPr>
@@ -2650,7 +2917,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">실행 클래스 안에서 순서대로 부르면 결과는 같지만</t>
+      <t xml:space="preserve">안 되면 실행 클래스 안에서 순차 호출이고</t>
     </r>
     <r>
       <rPr>
@@ -2667,7 +2934,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">스텝별 상태</t>
+      <t xml:space="preserve">그 경우 스텝별 상태</t>
     </r>
     <r>
       <rPr>
@@ -2701,7 +2968,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">재시작은 못 한다</t>
+      <t xml:space="preserve">재시작을 잃는다</t>
     </r>
   </si>
   <si>
@@ -4408,16 +4675,42 @@
     <t xml:space="preserve">step_nr</t>
   </si>
   <si>
-    <t xml:space="preserve">이 값이 붙을 스텝 번호</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">잡을 걸 때는 항상 </t>
+    <t xml:space="preserve">이 값이 붙을 단계 번호</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ADT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설명상 다단계 잡을 위한 필드다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스텝이 하나면 </t>
     </r>
     <r>
       <rPr>
@@ -4434,75 +4727,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">이다 — 스텝이 하나뿐이라 다른 값이 나올 수 없다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">필드가 있는 것은 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">APJ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">밖에서 만든 클래식 잡</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">스텝 여럿</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">을 읽을 때 같은 구조를 쓰기 때문으로 보인다</t>
+      <t xml:space="preserve">을 넣는다</t>
     </r>
     <r>
       <rPr>
@@ -6282,7 +6507,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6298,7 +6523,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E2F3"/>
-        <bgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -6310,7 +6535,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6E0B4"/>
-        <bgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -6328,6 +6553,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
         <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
@@ -6381,7 +6612,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6454,6 +6685,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6514,7 +6749,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FFC6E0B4"/>
       <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -6783,7 +7018,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
       <c r="B7" s="7" t="s">
         <v>12</v>
@@ -6791,10 +7026,10 @@
       <c r="C7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>15</v>
       </c>
     </row>
@@ -7074,74 +7309,74 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>73</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -7160,7 +7395,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7173,50 +7408,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">COUNTIF($E$8:$E$46,B4)</f>
         <v>11</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E4" s="14" t="n">
         <f aca="false">COUNTIF($E$8:$E$46,D4)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G4" s="14" t="n">
         <f aca="false">COUNTIF($E$8:$E$46,F4)</f>
         <v>11</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I4" s="14" t="n">
         <f aca="false">COUNTIF($E$8:$E$46,H4)</f>
         <v>6</v>
       </c>
+      <c r="J4" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <f aca="false">COUNTIF($E$8:$E$46,J4)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>96</v>
+      <c r="A5" s="19" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7224,24 +7466,24 @@
         <v>2</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -7252,78 +7494,78 @@
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
       <c r="B9" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
       <c r="B10" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>108</v>
+        <v>109</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
       <c r="B11" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>108</v>
+        <v>113</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
       <c r="B12" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>108</v>
+        <v>116</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -7331,128 +7573,128 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
       <c r="B14" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>108</v>
+        <v>120</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>121</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
       <c r="B15" s="7" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
       <c r="B16" s="8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
       <c r="B17" s="7" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
       <c r="B18" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>108</v>
+        <v>135</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
       <c r="B19" s="7" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
       <c r="B20" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>108</v>
+        <v>141</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7468,104 +7710,104 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
       <c r="B22" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6"/>
       <c r="B23" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
       <c r="B24" s="7" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6"/>
       <c r="B25" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>108</v>
+        <v>155</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6"/>
       <c r="B26" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>108</v>
+        <v>158</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6"/>
       <c r="B27" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>108</v>
+        <v>161</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F27" s="7"/>
     </row>
@@ -7582,112 +7824,112 @@
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6"/>
       <c r="B29" s="7" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6"/>
       <c r="B30" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>108</v>
+        <v>167</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6"/>
-      <c r="B31" s="19" t="s">
-        <v>108</v>
+      <c r="B31" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6"/>
-      <c r="B32" s="19" t="s">
-        <v>108</v>
+      <c r="B32" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6"/>
-      <c r="B33" s="19" t="s">
-        <v>108</v>
+      <c r="B33" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6"/>
-      <c r="B34" s="19" t="s">
-        <v>108</v>
+      <c r="B34" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -7698,94 +7940,94 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6"/>
       <c r="B36" s="7" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F36" s="7"/>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6"/>
       <c r="B37" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6"/>
       <c r="B38" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6"/>
       <c r="B39" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6"/>
       <c r="B40" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>108</v>
+        <v>197</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E40" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -7796,60 +8038,60 @@
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6"/>
       <c r="B42" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6"/>
       <c r="B43" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E43" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6"/>
       <c r="B44" s="7" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>208</v>
+        <v>93</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
@@ -7859,20 +8101,20 @@
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6"/>
-      <c r="B46" s="19" t="s">
-        <v>108</v>
+      <c r="B46" s="20" t="s">
+        <v>110</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -7911,107 +8153,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>215</v>
+      <c r="A4" s="21" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>237</v>
+      <c r="A11" s="21" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8019,21 +8261,21 @@
         <v>2</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -8043,51 +8285,51 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
       <c r="B14" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
       <c r="B15" s="8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
       <c r="B16" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -8097,21 +8339,21 @@
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
       <c r="B18" s="8" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>39</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -8121,56 +8363,56 @@
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
       <c r="B20" s="7" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6"/>
       <c r="B21" s="7" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
       <c r="B22" s="7" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>39</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
+      <c r="A24" s="22" t="s">
+        <v>270</v>
+      </c>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>